<commit_message>
SEQUOIADBMAINSTREAM-663: add queryandupdate & queryandremove to REST doc
git-svn-id: http://192.168.20.11/sequoiadb/trunk@18104 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
+++ b/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
   <si>
     <t>命令</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -251,6 +251,42 @@
   </si>
   <si>
     <t>curl http://192.168.20.197:50004/  -d "cmd=insert&amp;name=cs.cl&amp;insertor={"age":12, "name":\"hello\"}"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>queryandupdate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>queryandremove</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>查询更新</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>查询删除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandremove&amp;name=cs.cl&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={"name":\"hello\"}"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cmd：命令字; 
+name：cl名字;
+updator: 更新操作
+sort: 排序字段名
+selector: 查询结果列
+skip：跳过多少行
+returnnum：最大返回条数
+filter：查询条件
+returnnew:是否返回更新后记录</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandupdate&amp;name=cs.cl&amp;updator={"$inc":{age:1}}&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={"name":\"hello\"}"&amp;returnnew=true</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -361,74 +397,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -440,7 +408,7 @@
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="C7EDCC"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -717,12 +685,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="21.875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.75" style="2" customWidth="1"/>
     <col min="4" max="4" width="56.75" style="1" customWidth="1"/>
     <col min="5" max="5" width="10.25" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9" style="2"/>
@@ -847,121 +815,141 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="36">
+    <row r="8" spans="1:5" ht="108">
       <c r="A8" s="3" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="48">
+    <row r="9" spans="1:5" ht="84">
       <c r="A9" s="3" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="24">
+    <row r="10" spans="1:5" ht="36">
       <c r="A10" s="3" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="36">
+    <row r="11" spans="1:5" ht="48">
       <c r="A11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="24">
+      <c r="A12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="36">
+      <c r="A13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="72">
-      <c r="A12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="3"/>
+    <row r="14" spans="1:5" ht="72">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3"/>
@@ -980,9 +968,23 @@
     <row r="18" spans="1:5">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
SEQUOIADBMAINSTREAM-663: update queryandupdate of REST doc
git-svn-id: http://192.168.20.11/sequoiadb/trunk@18109 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
+++ b/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
@@ -276,7 +276,7 @@
   <si>
     <t>cmd：命令字; 
 name：cl名字;
-updator: 更新操作
+update: 更新操作
 sort: 排序字段名
 selector: 查询结果列
 skip：跳过多少行
@@ -286,7 +286,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandupdate&amp;name=cs.cl&amp;updator={"$inc":{age:1}}&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={"name":\"hello\"}"&amp;returnnew=true</t>
+    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandupdate&amp;name=cs.cl&amp;update={"$inc":{age:1}}&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={"name":\"hello\"}"&amp;returnnew=true</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
update queryandupdate of REST doc
git-svn-id: http://192.168.20.11/sequoiadb/trunk@18121 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
+++ b/internal_doc/03.开发设计/rest/sequoiadb引擎rest接口.xlsx
@@ -276,7 +276,7 @@
   <si>
     <t>cmd：命令字; 
 name：cl名字;
-update: 更新操作
+updator: 更新操作
 sort: 排序字段名
 selector: 查询结果列
 skip：跳过多少行
@@ -286,7 +286,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandupdate&amp;name=cs.cl&amp;update={"$inc":{age:1}}&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={"name":\"hello\"}"&amp;returnnew=true</t>
+    <t>curl http://192.168.20.197:50004/  -d "cmd=queryandupdate&amp;name=cs.cl&amp;updator={\"$inc\":{age:1}}&amp;sort={"name":null}&amp;skip=0&amp;returnnum=2&amp;filter={\"name\":\"hello\"}"&amp;returnnew=true</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>

</xml_diff>